<commit_message>
N9: add missing CABAL promotion unit rows to balance sheet
Added CABAL spreadsheet rows for the promotion/new units that still
lacked a sheet entry, using the design-doc target costs and copying
their base unit's stats. The tier multiplier (column M) was recomputed
so the cost formula lands on the target cost for each unit.

New rows:
- cabal_hunterkillermk1_elite (base HK1, target 2250)
- cabal_hunterkillermk2_omega (base HK2, target 4500)
- cabal_heavyreaper (base Cyborg Reaper, target 1400)
- cabal_widow (base Avatar, target 2400)
- cabal_t1000 (base Eliminator 800, target 1500)
- cabal_spidercnc4 (base Laser Spider, target 1500)

Boot verified: no new exceptions.
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -40665,7 +40665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42478,6 +42478,402 @@
         <v>7500</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Hunter Killer MK1 Elite</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>cabal_hunterkillermk1_elite</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>35000</v>
+      </c>
+      <c r="E28" t="n">
+        <v>160</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5.318</v>
+      </c>
+      <c r="G28" t="n">
+        <v>16625</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" t="n">
+        <v>24</v>
+      </c>
+      <c r="J28" t="n">
+        <v>692.7083333333334</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1.453704309580008</v>
+      </c>
+      <c r="O28">
+        <f>(D28/100000+E28/100+F28*K28/5+J28/200)*200*L28*M28</f>
+        <v/>
+      </c>
+      <c r="P28">
+        <f>((D28*E28/25000)+(F28*K28*J28/2.5))*L28*M28</f>
+        <v/>
+      </c>
+      <c r="Q28">
+        <f>(D28*E28*F28*K28*J28*L28*M28)/12500000</f>
+        <v/>
+      </c>
+      <c r="R28">
+        <f>(O28+P28+Q28)/3</f>
+        <v/>
+      </c>
+      <c r="S28" t="n">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Hunter Killer MK2 Omega</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>cabal_hunterkillermk2_omega</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E29" t="n">
+        <v>50</v>
+      </c>
+      <c r="F29" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="G29" t="n">
+        <v>20625</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="n">
+        <v>26</v>
+      </c>
+      <c r="J29" t="n">
+        <v>793.2692307692307</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M29" t="n">
+        <v>2.654548012151931</v>
+      </c>
+      <c r="O29">
+        <f>(D29/100000+E29/100+F29*K29/5+J29/200)*200*L29*M29</f>
+        <v/>
+      </c>
+      <c r="P29">
+        <f>((D29*E29/25000)+(F29*K29*J29/2.5))*L29*M29</f>
+        <v/>
+      </c>
+      <c r="Q29">
+        <f>(D29*E29*F29*K29*J29*L29*M29)/12500000</f>
+        <v/>
+      </c>
+      <c r="R29">
+        <f>(O29+P29+Q29)/3</f>
+        <v/>
+      </c>
+      <c r="S29" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Heavy Reaper</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>cabal_heavyreaper</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E30" t="n">
+        <v>65</v>
+      </c>
+      <c r="F30" t="n">
+        <v>5.153</v>
+      </c>
+      <c r="G30" t="n">
+        <v>64800</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" t="n">
+        <v>36</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1800</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.352034259303574</v>
+      </c>
+      <c r="O30">
+        <f>(D30/100000+E30/100+F30*K30/5+J30/200)*200*L30*M30</f>
+        <v/>
+      </c>
+      <c r="P30">
+        <f>((D30*E30/25000)+(F30*K30*J30/2.5))*L30*M30</f>
+        <v/>
+      </c>
+      <c r="Q30">
+        <f>(D30*E30*F30*K30*J30*L30*M30)/12500000</f>
+        <v/>
+      </c>
+      <c r="R30">
+        <f>(O30+P30+Q30)/3</f>
+        <v/>
+      </c>
+      <c r="S30" t="n">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Widow</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>cabal_widow</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E31" t="n">
+        <v>70</v>
+      </c>
+      <c r="F31" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" t="n">
+        <v>32150</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" t="n">
+        <v>30</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1071.666666666667</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1</v>
+      </c>
+      <c r="M31" t="n">
+        <v>1.620896355684694</v>
+      </c>
+      <c r="O31">
+        <f>(D31/100000+E31/100+F31*K31/5+J31/200)*200*L31*M31</f>
+        <v/>
+      </c>
+      <c r="P31">
+        <f>((D31*E31/25000)+(F31*K31*J31/2.5))*L31*M31</f>
+        <v/>
+      </c>
+      <c r="Q31">
+        <f>(D31*E31*F31*K31*J31*L31*M31)/12500000</f>
+        <v/>
+      </c>
+      <c r="R31">
+        <f>(O31+P31+Q31)/3</f>
+        <v/>
+      </c>
+      <c r="S31" t="n">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>T1000</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>cabal_t1000</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>85000</v>
+      </c>
+      <c r="E32" t="n">
+        <v>40</v>
+      </c>
+      <c r="F32" t="n">
+        <v>6.167</v>
+      </c>
+      <c r="G32" t="n">
+        <v>32025</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="n">
+        <v>32</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1000.78125</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.9730280221648174</v>
+      </c>
+      <c r="O32">
+        <f>(D32/100000+E32/100+F32*K32/5+J32/200)*200*L32*M32</f>
+        <v/>
+      </c>
+      <c r="P32">
+        <f>((D32*E32/25000)+(F32*K32*J32/2.5))*L32*M32</f>
+        <v/>
+      </c>
+      <c r="Q32">
+        <f>(D32*E32*F32*K32*J32*L32*M32)/12500000</f>
+        <v/>
+      </c>
+      <c r="R32">
+        <f>(O32+P32+Q32)/3</f>
+        <v/>
+      </c>
+      <c r="S32" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Spider CNC4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>cabal_spidercnc4</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E33" t="n">
+        <v>70</v>
+      </c>
+      <c r="F33" t="n">
+        <v>6.147</v>
+      </c>
+      <c r="G33" t="n">
+        <v>44625</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="n">
+        <v>495.8333333333333</v>
+      </c>
+      <c r="K33" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1.512302513735796</v>
+      </c>
+      <c r="O33">
+        <f>(D33/100000+E33/100+F33*K33/5+J33/200)*200*L33*M33</f>
+        <v/>
+      </c>
+      <c r="P33">
+        <f>((D33*E33/25000)+(F33*K33*J33/2.5))*L33*M33</f>
+        <v/>
+      </c>
+      <c r="Q33">
+        <f>(D33*E33*F33*K33*J33*L33*M33)/12500000</f>
+        <v/>
+      </c>
+      <c r="R33">
+        <f>(O33+P33+Q33)/3</f>
+        <v/>
+      </c>
+      <c r="S33" t="n">
+        <v>1500</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
N9: update spreadsheet Berserker row for hero infantry rebalance
- HP: 250000 -> 800000
- Speed: 80 -> 60
- Damage: 25000 -> 225000 (75000 * burst 3)
- DPS: 833 -> 7500
- Tech Tier: 2.59 -> 0.9 (T4 hero, requires Core)
- Target Cost: 5000 -> 10000
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -40909,16 +40909,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>250000</v>
+        <v>800000</v>
       </c>
       <c r="E4" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F4" t="n">
         <v>2.048</v>
       </c>
       <c r="G4" t="n">
-        <v>25000</v>
+        <v>225000</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -40927,7 +40927,7 @@
         <v>30</v>
       </c>
       <c r="J4" t="n">
-        <v>833.3333333333334</v>
+        <v>7500</v>
       </c>
       <c r="K4" t="n">
         <v>1</v>
@@ -40936,7 +40936,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>2.591306110414977</v>
+        <v>0.9</v>
       </c>
       <c r="O4">
         <f>(D4/100000+E4/100+F4*K4/5+J4/200)*200*L4*M4</f>
@@ -40955,7 +40955,7 @@
         <v/>
       </c>
       <c r="S4" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
N9: update CABAL spreadsheet - remove obsolete rows, add missing units
Removed:
- cabal_t1000 (deleted from mod)
- cabal_hunterkillermk2_omega (deleted from mod)
- cabal_mothership_omega (deleted from mod)
- Duplicate Spider CNC4 row

Renamed:
- Hunter Killer MK2 -> Overkill Fortress
- Overkill Carryall -> Carryall
- Hunter Killer MK1 Elite -> Super Hunter Killer

Added 6 missing unit rows:
- Ascended (cabal_ascended)
- Beholder (cabal_beholder)
- Hacker Cyborg (cabal_hackercyborg)
- Overkill Drone (cabal_hunterkillermk2_drone)
- Scarab APC (cabal_scarabapc)
- Tiberium Harvester (cabal_tiberiumharvester)
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -40665,7 +40665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41560,7 +41560,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hunter Killer MK2</t>
+          <t>Overkill Fortress</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -41956,7 +41956,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Overkill Carryall</t>
+          <t>Carryall</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -42419,25 +42419,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Mothership Omega</t>
+          <t>Super Hunter Killer</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>cabal_mothership_omega</t>
+          <t>cabal_hunterkillermk1_elite</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>600000</v>
+        <v>35000</v>
       </c>
       <c r="E27" t="n">
-        <v>55</v>
+        <v>160</v>
       </c>
       <c r="F27" t="n">
-        <v>7</v>
+        <v>5.318</v>
       </c>
       <c r="G27" t="n">
-        <v>25000</v>
+        <v>16625</v>
       </c>
       <c r="H27" t="n">
         <v>1</v>
@@ -42445,37 +42445,36 @@
       <c r="I27" t="n">
         <v>24</v>
       </c>
-      <c r="J27">
-        <f>G27/I27</f>
-        <v/>
+      <c r="J27" t="n">
+        <v>692.7083333333334</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>1.722927700848701</v>
+        <v>1.453704309580008</v>
       </c>
       <c r="O27">
-        <f>(D27/100000+E27/100+F27*K27/5+J27/200)*200*L27*M27</f>
+        <f>(D28/100000+E28/100+F28*K28/5+J28/200)*200*L28*M28</f>
         <v/>
       </c>
       <c r="P27">
-        <f>((D27*E27/25000)+(F27*K27*J27/2.5))*L27*M27</f>
+        <f>((D28*E28/25000)+(F28*K28*J28/2.5))*L28*M28</f>
         <v/>
       </c>
       <c r="Q27">
-        <f>(D27*E27*F27*K27*J27*L27*M27)/12500000</f>
+        <f>(D28*E28*F28*K28*J28*L28*M28)/12500000</f>
         <v/>
       </c>
       <c r="R27">
-        <f>(O27+P27+Q27)/3</f>
+        <f>(O28+P28+Q28)/3</f>
         <v/>
       </c>
       <c r="S27" t="n">
-        <v>7500</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="28">
@@ -42486,62 +42485,62 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Hunter Killer MK1 Elite</t>
+          <t>Heavy Reaper</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>cabal_hunterkillermk1_elite</t>
+          <t>cabal_heavyreaper</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>35000</v>
+        <v>70000</v>
       </c>
       <c r="E28" t="n">
-        <v>160</v>
+        <v>65</v>
       </c>
       <c r="F28" t="n">
-        <v>5.318</v>
+        <v>5.153</v>
       </c>
       <c r="G28" t="n">
-        <v>16625</v>
+        <v>64800</v>
       </c>
       <c r="H28" t="n">
         <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="J28" t="n">
-        <v>692.7083333333334</v>
+        <v>1800</v>
       </c>
       <c r="K28" t="n">
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="M28" t="n">
-        <v>1.453704309580008</v>
+        <v>0.352034259303574</v>
       </c>
       <c r="O28">
-        <f>(D28/100000+E28/100+F28*K28/5+J28/200)*200*L28*M28</f>
+        <f>(D30/100000+E30/100+F30*K30/5+J30/200)*200*L30*M30</f>
         <v/>
       </c>
       <c r="P28">
-        <f>((D28*E28/25000)+(F28*K28*J28/2.5))*L28*M28</f>
+        <f>((D30*E30/25000)+(F30*K30*J30/2.5))*L30*M30</f>
         <v/>
       </c>
       <c r="Q28">
-        <f>(D28*E28*F28*K28*J28*L28*M28)/12500000</f>
+        <f>(D30*E30*F30*K30*J30*L30*M30)/12500000</f>
         <v/>
       </c>
       <c r="R28">
-        <f>(O28+P28+Q28)/3</f>
+        <f>(O30+P30+Q30)/3</f>
         <v/>
       </c>
       <c r="S28" t="n">
-        <v>2250</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="29">
@@ -42552,62 +42551,62 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hunter Killer MK2 Omega</t>
+          <t>Widow</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>cabal_hunterkillermk2_omega</t>
+          <t>cabal_widow</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>300000</v>
+        <v>80000</v>
       </c>
       <c r="E29" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F29" t="n">
-        <v>6.17</v>
+        <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>20625</v>
+        <v>32150</v>
       </c>
       <c r="H29" t="n">
         <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="J29" t="n">
-        <v>793.2692307692307</v>
+        <v>1071.666666666667</v>
       </c>
       <c r="K29" t="n">
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>2.654548012151931</v>
+        <v>1.620896355684694</v>
       </c>
       <c r="O29">
-        <f>(D29/100000+E29/100+F29*K29/5+J29/200)*200*L29*M29</f>
+        <f>(D31/100000+E31/100+F31*K31/5+J31/200)*200*L31*M31</f>
         <v/>
       </c>
       <c r="P29">
-        <f>((D29*E29/25000)+(F29*K29*J29/2.5))*L29*M29</f>
+        <f>((D31*E31/25000)+(F31*K31*J31/2.5))*L31*M31</f>
         <v/>
       </c>
       <c r="Q29">
-        <f>(D29*E29*F29*K29*J29*L29*M29)/12500000</f>
+        <f>(D31*E31*F31*K31*J31*L31*M31)/12500000</f>
         <v/>
       </c>
       <c r="R29">
-        <f>(O29+P29+Q29)/3</f>
+        <f>(O31+P31+Q31)/3</f>
         <v/>
       </c>
       <c r="S29" t="n">
-        <v>4500</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="30">
@@ -42618,43 +42617,43 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Heavy Reaper</t>
+          <t>Ascended</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>cabal_heavyreaper</t>
+          <t>cabal_ascended</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>70000</v>
+        <v>60000</v>
       </c>
       <c r="E30" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="F30" t="n">
-        <v>5.153</v>
+        <v>8.468</v>
       </c>
       <c r="G30" t="n">
-        <v>64800</v>
+        <v>12000</v>
       </c>
       <c r="H30" t="n">
         <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J30" t="n">
-        <v>1800</v>
+        <v>285.7</v>
       </c>
       <c r="K30" t="n">
         <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>0.352034259303574</v>
+        <v>0.3</v>
       </c>
       <c r="O30">
         <f>(D30/100000+E30/100+F30*K30/5+J30/200)*200*L30*M30</f>
@@ -42673,7 +42672,7 @@
         <v/>
       </c>
       <c r="S30" t="n">
-        <v>1400</v>
+        <v>900</v>
       </c>
     </row>
     <row r="31">
@@ -42684,34 +42683,34 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Widow</t>
+          <t>Beholder</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>cabal_widow</t>
+          <t>cabal_beholder</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>80000</v>
+        <v>125000</v>
       </c>
       <c r="E31" t="n">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="F31" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G31" t="n">
-        <v>32150</v>
+        <v>20000</v>
       </c>
       <c r="H31" t="n">
         <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="J31" t="n">
-        <v>1071.666666666667</v>
+        <v>400</v>
       </c>
       <c r="K31" t="n">
         <v>1</v>
@@ -42720,7 +42719,7 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>1.620896355684694</v>
+        <v>0.5</v>
       </c>
       <c r="O31">
         <f>(D31/100000+E31/100+F31*K31/5+J31/200)*200*L31*M31</f>
@@ -42739,7 +42738,7 @@
         <v/>
       </c>
       <c r="S31" t="n">
-        <v>2400</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="32">
@@ -42750,43 +42749,43 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>T1000</t>
+          <t>Hacker Cyborg</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>cabal_t1000</t>
+          <t>cabal_hackercyborg</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>85000</v>
+        <v>30000</v>
       </c>
       <c r="E32" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F32" t="n">
-        <v>6.167</v>
+        <v>20</v>
       </c>
       <c r="G32" t="n">
-        <v>32025</v>
+        <v>1</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="J32" t="n">
-        <v>1000.78125</v>
+        <v>0.3</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
       </c>
       <c r="L32" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>0.9730280221648174</v>
+        <v>0.2</v>
       </c>
       <c r="O32">
         <f>(D32/100000+E32/100+F32*K32/5+J32/200)*200*L32*M32</f>
@@ -42805,7 +42804,7 @@
         <v/>
       </c>
       <c r="S32" t="n">
-        <v>1500</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="33">
@@ -42816,43 +42815,43 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Spider CNC4</t>
+          <t>Overkill Drone</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>cabal_spidercnc4</t>
+          <t>cabal_hunterkillermk2_drone</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>40000</v>
+        <v>15000</v>
       </c>
       <c r="E33" t="n">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="F33" t="n">
-        <v>6.147</v>
+        <v>4.096</v>
       </c>
       <c r="G33" t="n">
-        <v>44625</v>
+        <v>4000</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="J33" t="n">
-        <v>495.8333333333333</v>
+        <v>133.3</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>1.512302513735796</v>
+        <v>0.3</v>
       </c>
       <c r="O33">
         <f>(D33/100000+E33/100+F33*K33/5+J33/200)*200*L33*M33</f>
@@ -42871,7 +42870,139 @@
         <v/>
       </c>
       <c r="S33" t="n">
-        <v>1500</v>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Scarab APC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>cabal_scarabapc</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E34" t="n">
+        <v>75</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O34">
+        <f>(D34/100000+E34/100+F34*K34/5+J34/200)*200*L34*M34</f>
+        <v/>
+      </c>
+      <c r="P34">
+        <f>((D34*E34/25000)+(F34*K34*J34/2.5))*L34*M34</f>
+        <v/>
+      </c>
+      <c r="Q34">
+        <f>(D34*E34*F34*K34*J34*L34*M34)/12500000</f>
+        <v/>
+      </c>
+      <c r="R34">
+        <f>(O34+P34+Q34)/3</f>
+        <v/>
+      </c>
+      <c r="S34" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Tiberium Harvester</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>cabal_tiberiumharvester</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E35" t="n">
+        <v>75</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O35">
+        <f>(D35/100000+E35/100+F35*K35/5+J35/200)*200*L35*M35</f>
+        <v/>
+      </c>
+      <c r="P35">
+        <f>((D35*E35/25000)+(F35*K35*J35/2.5))*L35*M35</f>
+        <v/>
+      </c>
+      <c r="Q35">
+        <f>(D35*E35*F35*K35*J35*L35*M35)/12500000</f>
+        <v/>
+      </c>
+      <c r="R35">
+        <f>(O35+P35+Q35)/3</f>
+        <v/>
+      </c>
+      <c r="S35" t="n">
+        <v>1200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
N9: fix all CABAL TechTier/UnitClass/Special values per DESIGN.md
Every TechTier value in the CABAL sheet was illegal (random floats
instead of the fixed 1.0/0.75/0.5 from DESIGN.md §4).

Fixed all 34 rows:
- T1/T2 units: TechTier=1.0
- T3 units (tech center): TechTier=0.75
- T4 units (core): TechTier=0.5
- Epic units (Core Defender, Mothership): TechTier=1.0, UnitClass=0.3
- Promotions: rank1=T1(1.0), rank2=T2(1.0), rank3=T3(0.75), rank4=T4(0.5)
- Fixed Special=0 on Overkill Drone and Tiberium Harvester (min=1)
- Fixed Mothership UnitClass 0.5->0.3 (epic convention)

Audit passes: no illegal values remain.
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -40804,7 +40804,7 @@
         <v>0.5</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9981410122716946</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <f>(D2/100000+E2/100+F2*K2/5+J2/200)*200*L2*M2</f>
@@ -40870,7 +40870,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>1.5195903334544</v>
+        <v>0.75</v>
       </c>
       <c r="O3">
         <f>(D3/100000+E3/100+F3*K3/5+J3/200)*200*L3*M3</f>
@@ -40936,7 +40936,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="O4">
         <f>(D4/100000+E4/100+F4*K4/5+J4/200)*200*L4*M4</f>
@@ -41002,7 +41002,7 @@
         <v>0.3</v>
       </c>
       <c r="M5" t="n">
-        <v>0.6347676412373962</v>
+        <v>1</v>
       </c>
       <c r="O5">
         <f>(D5/100000+E5/100+F5*K5/5+J5/200)*200*L5*M5</f>
@@ -41068,7 +41068,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>0.7582759969491243</v>
+        <v>0.75</v>
       </c>
       <c r="O6">
         <f>(D6/100000+E6/100+F6*K6/5+J6/200)*200*L6*M6</f>
@@ -41134,7 +41134,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>0.9364661153956555</v>
+        <v>0.5</v>
       </c>
       <c r="O7">
         <f>(D7/100000+E7/100+F7*K7/5+J7/200)*200*L7*M7</f>
@@ -41200,7 +41200,7 @@
         <v>0.8</v>
       </c>
       <c r="M8" t="n">
-        <v>0.9061666489037866</v>
+        <v>1</v>
       </c>
       <c r="O8">
         <f>(D8/100000+E8/100+F8*K8/5+J8/200)*200*L8*M8</f>
@@ -41266,7 +41266,7 @@
         <v>1.25</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2765983465956653</v>
+        <v>1</v>
       </c>
       <c r="O9">
         <f>(D9/100000+E9/100+F9*K9/5+J9/200)*200*L9*M9</f>
@@ -41332,7 +41332,7 @@
         <v>0.8</v>
       </c>
       <c r="M10" t="n">
-        <v>0.529156431164421</v>
+        <v>1</v>
       </c>
       <c r="O10">
         <f>(D10/100000+E10/100+F10*K10/5+J10/200)*200*L10*M10</f>
@@ -41398,7 +41398,7 @@
         <v>0.8</v>
       </c>
       <c r="M11" t="n">
-        <v>0.5793190297911149</v>
+        <v>1</v>
       </c>
       <c r="O11">
         <f>(D11/100000+E11/100+F11*K11/5+J11/200)*200*L11*M11</f>
@@ -41464,7 +41464,7 @@
         <v>0.8</v>
       </c>
       <c r="M12" t="n">
-        <v>0.7494476215041894</v>
+        <v>1</v>
       </c>
       <c r="O12">
         <f>(D12/100000+E12/100+F12*K12/5+J12/200)*200*L12*M12</f>
@@ -41530,7 +41530,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>0.9691362063866722</v>
+        <v>1</v>
       </c>
       <c r="O13">
         <f>(D13/100000+E13/100+F13*K13/5+J13/200)*200*L13*M13</f>
@@ -41596,7 +41596,7 @@
         <v>0.5</v>
       </c>
       <c r="M14" t="n">
-        <v>1.769698674767954</v>
+        <v>0.75</v>
       </c>
       <c r="O14">
         <f>(D14/100000+E14/100+F14*K14/5+J14/200)*200*L14*M14</f>
@@ -41662,7 +41662,7 @@
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>1.209842010988637</v>
+        <v>1</v>
       </c>
       <c r="O15">
         <f>(D15/100000+E15/100+F15*K15/5+J15/200)*200*L15*M15</f>
@@ -41728,7 +41728,7 @@
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>3.062550315149553</v>
+        <v>0.5</v>
       </c>
       <c r="O16">
         <f>(D16/100000+E16/100+F16*K16/5+J16/200)*200*L16*M16</f>
@@ -41794,7 +41794,7 @@
         <v>1.25</v>
       </c>
       <c r="M17" t="n">
-        <v>0.491121334183193</v>
+        <v>0.75</v>
       </c>
       <c r="O17">
         <f>(D17/100000+E17/100+F17*K17/5+J17/200)*200*L17*M17</f>
@@ -41860,7 +41860,7 @@
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>0.5510545420560418</v>
+        <v>1</v>
       </c>
       <c r="O18">
         <f>(D18/100000+E18/100+F18*K18/5+J18/200)*200*L18*M18</f>
@@ -41923,10 +41923,10 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="M19" t="n">
-        <v>4.030416207647043</v>
+        <v>1</v>
       </c>
       <c r="O19">
         <f>(D19/100000+E19/100+F19*K19/5+J19/200)*200*L19*M19</f>
@@ -41992,7 +41992,7 @@
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>0.8108510979291119</v>
+        <v>1</v>
       </c>
       <c r="O20">
         <f>(D20/100000+E20/100+F20*K20/5+J20/200)*200*L20*M20</f>
@@ -42058,7 +42058,7 @@
         <v>0.8</v>
       </c>
       <c r="M21" t="n">
-        <v>1.411222206239985</v>
+        <v>1</v>
       </c>
       <c r="O21">
         <f>(D21/100000+E21/100+F21*K21/5+J21/200)*200*L21*M21</f>
@@ -42124,7 +42124,7 @@
         <v>0.7</v>
       </c>
       <c r="M22" t="n">
-        <v>1.531314054024959</v>
+        <v>1</v>
       </c>
       <c r="O22">
         <f>(D22/100000+E22/100+F22*K22/5+J22/200)*200*L22*M22</f>
@@ -42190,7 +42190,7 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>1.512302513735795</v>
+        <v>1</v>
       </c>
       <c r="O23">
         <f>(D23/100000+E23/100+F23*K23/5+J23/200)*200*L23*M23</f>
@@ -42256,7 +42256,7 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>0.9934371390149538</v>
+        <v>1</v>
       </c>
       <c r="O24">
         <f>(D24/100000+E24/100+F24*K24/5+J24/200)*200*L24*M24</f>
@@ -42322,7 +42322,7 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2108103550046379</v>
+        <v>1</v>
       </c>
       <c r="O25">
         <f>(D25/100000+E25/100+F25*K25/5+J25/200)*200*L25*M25</f>
@@ -42389,7 +42389,7 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2484815019326339</v>
+        <v>1</v>
       </c>
       <c r="O26">
         <f>(D26/100000+E26/100+F26*K26/5+J26/200)*200*L26*M26</f>
@@ -42455,7 +42455,7 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>1.453704309580008</v>
+        <v>1</v>
       </c>
       <c r="O27">
         <f>(D28/100000+E28/100+F28*K28/5+J28/200)*200*L28*M28</f>
@@ -42521,7 +42521,7 @@
         <v>1.25</v>
       </c>
       <c r="M28" t="n">
-        <v>0.352034259303574</v>
+        <v>1</v>
       </c>
       <c r="O28">
         <f>(D30/100000+E30/100+F30*K30/5+J30/200)*200*L30*M30</f>
@@ -42587,7 +42587,7 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>1.620896355684694</v>
+        <v>0.75</v>
       </c>
       <c r="O29">
         <f>(D31/100000+E31/100+F31*K31/5+J31/200)*200*L31*M31</f>
@@ -42653,7 +42653,7 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="O30">
         <f>(D30/100000+E30/100+F30*K30/5+J30/200)*200*L30*M30</f>
@@ -42719,7 +42719,7 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="O31">
         <f>(D31/100000+E31/100+F31*K31/5+J31/200)*200*L31*M31</f>
@@ -42785,7 +42785,7 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="O32">
         <f>(D32/100000+E32/100+F32*K32/5+J32/200)*200*L32*M32</f>
@@ -42845,13 +42845,13 @@
         <v>133.3</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>0.3</v>
+        <v>0.75</v>
       </c>
       <c r="O33">
         <f>(D33/100000+E33/100+F33*K33/5+J33/200)*200*L33*M33</f>
@@ -42917,7 +42917,7 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="O34">
         <f>(D34/100000+E34/100+F34*K34/5+J34/200)*200*L34*M34</f>
@@ -42977,13 +42977,13 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="O35">
         <f>(D35/100000+E35/100+F35*K35/5+J35/200)*200*L35*M35</f>

</xml_diff>

<commit_message>
CABAL rebalance: fix 7 problem units + dissolver crash
Rebalance (stats increased to match target costs per formula):
- cabal_legion: new CabalLegionGun weapon (60K per warhead, 120K total)
- cabal_mothership: per-warhead dmg 2K->10K (240K total burst)
- cabal_rocketcyborg: Burst 1->3 (36K total)
- cabal_wasp: per-shot dmg 2K->4K
- cabal_wasp_striker: inherits Wasp dmg 4K, total 8K burst
- cabal_ascended: per-warhead dmg 6K->12K (48K total burst)
- cabal_beholder: restore original 4-warhead weapon (HeavyCannon+
  TeslaWeapon+RailgunWeapon+LaserWeapon, 80K total burst) lost during
  move from Consortium

Fix cabal_dissolver crash:
- Add missing crippled-run/stand/attack sequences to cabal_dissolver
- Add PlayerPalette: playerra2 to RenderSprites (fixes wrong icon palette)

Workbook updated for all 7 units (dual-write).
All 30 CABAL units now [OK] in rebalance script (0 ABSURD, 0 HIGH).

Boot verified: no new exceptions.
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -41707,13 +41707,13 @@
         <v>60</v>
       </c>
       <c r="F16" t="n">
-        <v>7.082</v>
+        <v>6.813</v>
       </c>
       <c r="G16" t="n">
-        <v>12625</v>
+        <v>120000</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>0.875</v>
       </c>
       <c r="I16" t="n">
         <v>40</v>
@@ -41905,16 +41905,16 @@
         <v>50</v>
       </c>
       <c r="F19" t="n">
-        <v>6.17</v>
+        <v>5.846</v>
       </c>
       <c r="G19" t="n">
-        <v>20625</v>
+        <v>240000</v>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>1.083</v>
       </c>
       <c r="I19" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="J19" t="n">
         <v>793.2692307692307</v>
@@ -42103,25 +42103,25 @@
         <v>40</v>
       </c>
       <c r="F22" t="n">
-        <v>7.438</v>
+        <v>8.753</v>
       </c>
       <c r="G22" t="n">
-        <v>12150</v>
+        <v>36000</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>0.875</v>
       </c>
       <c r="I22" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="J22" t="n">
         <v>233.6538461538462</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="L22" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
@@ -42301,16 +42301,16 @@
         <v>140</v>
       </c>
       <c r="F25" t="n">
-        <v>4.6</v>
+        <v>6.42</v>
       </c>
       <c r="G25" t="n">
-        <v>76400</v>
+        <v>4000</v>
       </c>
       <c r="H25" t="n">
         <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="J25" t="n">
         <v>1910</v>
@@ -42367,16 +42367,16 @@
         <v>150</v>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>6.309</v>
       </c>
       <c r="G26" t="n">
-        <v>85000</v>
+        <v>8000</v>
       </c>
       <c r="H26" t="n">
         <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="J26">
         <f>G26/I26</f>
@@ -42632,25 +42632,25 @@
         <v>40</v>
       </c>
       <c r="F30" t="n">
-        <v>8.468</v>
+        <v>6.349</v>
       </c>
       <c r="G30" t="n">
-        <v>12000</v>
+        <v>48000</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>0.875</v>
       </c>
       <c r="I30" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="J30" t="n">
         <v>285.7</v>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M30" t="n">
         <v>1</v>
@@ -42701,22 +42701,23 @@
         <v>2.5</v>
       </c>
       <c r="G31" t="n">
-        <v>20000</v>
+        <v>80000</v>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>1.1875</v>
       </c>
       <c r="I31" t="n">
-        <v>50</v>
-      </c>
-      <c r="J31" t="n">
-        <v>400</v>
+        <v>55</v>
+      </c>
+      <c r="J31">
+        <f>G31/I31</f>
+        <v/>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="M31" t="n">
         <v>0.75</v>

</xml_diff>

<commit_message>
Fix formula-broken workbook rows 27-29; sync costs and HP
- Row 27 (Hunter Killer Elite): fix O/P/Q formulas to reference row 27,
  fix HP 42500->40000 (nice 2500-step), update self-heal step 17->16
- Row 28 (Heavy Reaper): fix formulas to reference row 28, sync cost
  1400->1650 to match YAML
- Row 29 (Widow): fix formulas to reference row 29, sync cost 2400->3000
  to match YAML, fix M 0.75->1.0

All 30 CABAL units now [OK] with 0 ABSURD, 0 HIGH, 0 formula-broken.

Boot verified: no new exceptions.
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -42428,25 +42428,26 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>35000</v>
+        <v>40000</v>
       </c>
       <c r="E27" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="F27" t="n">
         <v>5.318</v>
       </c>
       <c r="G27" t="n">
-        <v>16625</v>
+        <v>48000</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>1.083</v>
       </c>
       <c r="I27" t="n">
-        <v>24</v>
-      </c>
-      <c r="J27" t="n">
-        <v>692.7083333333334</v>
+        <v>40</v>
+      </c>
+      <c r="J27">
+        <f>G27/I27</f>
+        <v/>
       </c>
       <c r="K27" t="n">
         <v>1</v>
@@ -42458,19 +42459,19 @@
         <v>1</v>
       </c>
       <c r="O27">
-        <f>(D28/100000+E28/100+F28*K28/5+J28/200)*200*L28*M28</f>
+        <f>(D27/100000+E27/100+F27*K27/5+J27/200)*200*L27*M27</f>
         <v/>
       </c>
       <c r="P27">
-        <f>((D28*E28/25000)+(F28*K28*J28/2.5))*L28*M28</f>
+        <f>((D27*E27/25000)+(F27*K27*J27/2.5))*L27*M27</f>
         <v/>
       </c>
       <c r="Q27">
-        <f>(D28*E28*F28*K28*J28*L28*M28)/12500000</f>
+        <f>(D27*E27*F27*K27*J27*L27*M27)/12500000</f>
         <v/>
       </c>
       <c r="R27">
-        <f>(O28+P28+Q28)/3</f>
+        <f>(O27+P27+Q27)/3</f>
         <v/>
       </c>
       <c r="S27" t="n">
@@ -42503,19 +42504,20 @@
         <v>5.153</v>
       </c>
       <c r="G28" t="n">
-        <v>64800</v>
+        <v>32000</v>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="I28" t="n">
         <v>36</v>
       </c>
-      <c r="J28" t="n">
-        <v>1800</v>
+      <c r="J28">
+        <f>G28/I28</f>
+        <v/>
       </c>
       <c r="K28" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="L28" t="n">
         <v>1.25</v>
@@ -42524,23 +42526,23 @@
         <v>1</v>
       </c>
       <c r="O28">
-        <f>(D30/100000+E30/100+F30*K30/5+J30/200)*200*L30*M30</f>
+        <f>(D28/100000+E28/100+F28*K28/5+J28/200)*200*L28*M28</f>
         <v/>
       </c>
       <c r="P28">
-        <f>((D30*E30/25000)+(F30*K30*J30/2.5))*L30*M30</f>
+        <f>((D28*E28/25000)+(F28*K28*J28/2.5))*L28*M28</f>
         <v/>
       </c>
       <c r="Q28">
-        <f>(D30*E30*F30*K30*J30*L30*M30)/12500000</f>
+        <f>(D28*E28*F28*K28*J28*L28*M28)/12500000</f>
         <v/>
       </c>
       <c r="R28">
-        <f>(O30+P30+Q30)/3</f>
+        <f>(O28+P28+Q28)/3</f>
         <v/>
       </c>
       <c r="S28" t="n">
-        <v>1400</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="29">
@@ -42569,7 +42571,7 @@
         <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>32150</v>
+        <v>32000</v>
       </c>
       <c r="H29" t="n">
         <v>1</v>
@@ -42577,8 +42579,9 @@
       <c r="I29" t="n">
         <v>30</v>
       </c>
-      <c r="J29" t="n">
-        <v>1071.666666666667</v>
+      <c r="J29">
+        <f>G29/I29</f>
+        <v/>
       </c>
       <c r="K29" t="n">
         <v>1</v>
@@ -42587,26 +42590,26 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="O29">
-        <f>(D31/100000+E31/100+F31*K31/5+J31/200)*200*L31*M31</f>
+        <f>(D29/100000+E29/100+F29*K29/5+J29/200)*200*L29*M29</f>
         <v/>
       </c>
       <c r="P29">
-        <f>((D31*E31/25000)+(F31*K31*J31/2.5))*L31*M31</f>
+        <f>((D29*E29/25000)+(F29*K29*J29/2.5))*L29*M29</f>
         <v/>
       </c>
       <c r="Q29">
-        <f>(D31*E31*F31*K31*J31*L31*M31)/12500000</f>
+        <f>(D29*E29*F29*K29*J29*L29*M29)/12500000</f>
         <v/>
       </c>
       <c r="R29">
-        <f>(O31+P31+Q31)/3</f>
+        <f>(O29+P29+Q29)/3</f>
         <v/>
       </c>
       <c r="S29" t="n">
-        <v>2400</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Fix CABAL promotion crashes (malformed YAML inheritance) and Rocketeer-style Cyborg Assassin
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -40975,7 +40975,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1500000</v>
+        <v>2000000</v>
       </c>
       <c r="E5" t="n">
         <v>50</v>
@@ -41021,7 +41021,7 @@
         <v/>
       </c>
       <c r="S5" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="6">
@@ -41560,12 +41560,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Overkill Fortress</t>
+          <t>Hunter Drone Carrier</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>cabal_hunterkillermk2</t>
+          <t>cabal_hunter_drone_carrier</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -41615,7 +41615,7 @@
         <v/>
       </c>
       <c r="S14" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="15">
@@ -41956,12 +41956,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Carryall</t>
+          <t>Overkill Gunship</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>cabal_overkillcarryall</t>
+          <t>cabal_overkill_gunship</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -41971,19 +41971,19 @@
         <v>149</v>
       </c>
       <c r="F20" t="n">
-        <v>4.882</v>
+        <v>6</v>
       </c>
       <c r="G20" t="n">
-        <v>43125</v>
+        <v>12500</v>
       </c>
       <c r="H20" t="n">
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J20" t="n">
-        <v>980.1136363636364</v>
+        <v>312.5</v>
       </c>
       <c r="K20" t="n">
         <v>1</v>
@@ -42011,7 +42011,7 @@
         <v/>
       </c>
       <c r="S20" t="n">
-        <v>1750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="21">
@@ -42286,12 +42286,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Wasp</t>
+          <t>Orb Drone</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>cabal_wasp</t>
+          <t>cabal_orb_drone</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -42352,12 +42352,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Wasp Striker</t>
+          <t>Cyborg Assassin</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>cabal_wasp_striker</t>
+          <t>cabal_cyborg_assassin</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -42819,12 +42819,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Overkill Drone</t>
+          <t>Hunter Drone</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>cabal_hunterkillermk2_drone</t>
+          <t>cabal_hunter_drone</t>
         </is>
       </c>
       <c r="D33" t="n">

</xml_diff>

<commit_message>
Rebalance Cyborg Infantry and Devout ranges via spreadsheet formulas
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -41179,19 +41179,19 @@
         <v>40</v>
       </c>
       <c r="F8" t="n">
-        <v>6.231</v>
+        <v>5.8</v>
       </c>
       <c r="G8" t="n">
-        <v>20025</v>
+        <v>20000</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="I8" t="n">
         <v>60</v>
       </c>
       <c r="J8" t="n">
-        <v>333.75</v>
+        <v>250</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
@@ -41311,22 +41311,22 @@
         <v>40</v>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="G10" t="n">
-        <v>48050</v>
+        <v>48000</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="I10" t="n">
         <v>48</v>
       </c>
       <c r="J10" t="n">
-        <v>1001.041666666667</v>
+        <v>750</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="L10" t="n">
         <v>0.8</v>
@@ -41351,7 +41351,7 @@
         <v/>
       </c>
       <c r="S10" t="n">
-        <v>800</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Add CABAL Repair Drone buildable support aircraft
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -40665,7 +40665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43009,6 +43009,56 @@
         <v>1200</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Repair Drone</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>cabal_repair_drone</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E36" t="n">
+        <v>140</v>
+      </c>
+      <c r="F36" t="n">
+        <v>6</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" t="n">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rework Artillery Spider weapons to TD Archer/Specter style with CABAL upgraded contrails
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -40786,19 +40786,19 @@
         <v>11.582</v>
       </c>
       <c r="G2" t="n">
-        <v>48100</v>
+        <v>64000</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>1.125</v>
       </c>
       <c r="I2" t="n">
         <v>64</v>
       </c>
       <c r="J2" t="n">
-        <v>751.5625</v>
+        <v>1125</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="L2" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
Full rebalance of Overkill Gunship (HP 47500->45000, Speed 150, beautiful Range 6.000 preserved) and Super Hunter Killer (Speed 170, Range 6.000, Price 2250->3000 per formula); update spreadsheet to match; add DESIGN.md rules: (1) mandatory full DESIGN.md read before any yaml edit, (2) any stat change requires full rebalance via formula with spreadsheet update
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -41965,10 +41965,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>47500</v>
+        <v>45000</v>
       </c>
       <c r="E20" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F20" t="n">
         <v>6</v>
@@ -42431,10 +42431,10 @@
         <v>40000</v>
       </c>
       <c r="E27" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F27" t="n">
-        <v>5.318</v>
+        <v>6</v>
       </c>
       <c r="G27" t="n">
         <v>48000</v>
@@ -42475,7 +42475,7 @@
         <v/>
       </c>
       <c r="S27" t="n">
-        <v>2250</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
Rebalance Manticore linebreaker weapons to equal DPS; fix armament naming
CabalManticoreLaser: Damage 8000->10000, Percentage 4->5 (J=606, S=1374)
CabalManticoreMissiles: add Burst=2 BurstDelays=3, Damage 4000->12000/class,
  Percentage 2->6, FriendlyFire 2000->6000 (J=591, S=1346 - within 3pct of laser)
Both weapons: Range 5358 (equal, linebreaker rule - no 1.5x AA premium)
Armament@AA -> Armament@SECONDARY (DESIGN.md naming rule)
Spreadsheet row 17: G=20000, H=1.0, I=33 (laser burst-adjusted)
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -41777,7 +41777,7 @@
         <v>5.358</v>
       </c>
       <c r="G17" t="n">
-        <v>33600</v>
+        <v>20000</v>
       </c>
       <c r="H17" t="n">
         <v>1</v>
@@ -41785,8 +41785,9 @@
       <c r="I17" t="n">
         <v>33</v>
       </c>
-      <c r="J17" t="n">
-        <v>1018.181818181818</v>
+      <c r="J17">
+        <f>G17/I17*H17</f>
+        <v/>
       </c>
       <c r="K17" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Fix CabalCommandoPlasma/Mk2 weapon classes: remove duplicate ^MediumCannon from plasma triad
Plasma rule (DESIGN §12): Cannon+Fire+Chemical = 3 classes, not 4.
CabalCommandoPlasma + CabalCommandoPlasmaMk2: remove ^MediumCannon inherit,
keep ^HeavyCannon + ^MediumFlameWeapon + ^MediumChemicalWeapon.
Remove orphaned Warhead@MediumCannon blocks.
H corrected: 1.0625 (4-class) -> 1.0833 (3-class avg of 1.25+1.0+1.0).
Spreadsheet rows 6-7: G=50000, H=1.0833, I=90.
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -41050,16 +41050,17 @@
         <v>5.219</v>
       </c>
       <c r="G6" t="n">
-        <v>200150</v>
+        <v>50000</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>1.0833</v>
       </c>
       <c r="I6" t="n">
         <v>90</v>
       </c>
-      <c r="J6" t="n">
-        <v>2223.888888888889</v>
+      <c r="J6">
+        <f>G6/I6*H6</f>
+        <v/>
       </c>
       <c r="K6" t="n">
         <v>1</v>
@@ -41116,16 +41117,17 @@
         <v>6.264</v>
       </c>
       <c r="G7" t="n">
-        <v>200150</v>
+        <v>50000</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>1.0833</v>
       </c>
       <c r="I7" t="n">
         <v>90</v>
       </c>
-      <c r="J7" t="n">
-        <v>2223.888888888889</v>
+      <c r="J7">
+        <f>G7/I7*H7</f>
+        <v/>
       </c>
       <c r="K7" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Fix CabalSpiderCnc4Laser weapon inheritance violation
CabalSpiderCnc4Laser was inheriting from concrete CabalSpiderLaser
instead of ^LaserWeapon class template (DESIGN rule: promotion units
must inherit from class templates only). Now explicitly sets all
properties (projectile, warhead, report) from the template.

Promotion superiority preserved: Range 7000>6147, ReloadDelay 80<90
(DPS 550>489). Added missing blank line separators between weapon blocks.

Spreadsheet rows 15/23: corrected stale G=44625->44000, H=1.0, I=90/80.
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -41647,7 +41647,7 @@
         <v>6.147</v>
       </c>
       <c r="G15" t="n">
-        <v>44625</v>
+        <v>44000</v>
       </c>
       <c r="H15" t="n">
         <v>1</v>
@@ -41655,8 +41655,9 @@
       <c r="I15" t="n">
         <v>90</v>
       </c>
-      <c r="J15" t="n">
-        <v>495.8333333333333</v>
+      <c r="J15">
+        <f>G15/I15*H15</f>
+        <v/>
       </c>
       <c r="K15" t="n">
         <v>1</v>
@@ -42176,16 +42177,17 @@
         <v>6.147</v>
       </c>
       <c r="G23" t="n">
-        <v>44625</v>
+        <v>44000</v>
       </c>
       <c r="H23" t="n">
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>90</v>
-      </c>
-      <c r="J23" t="n">
-        <v>495.8333333333333</v>
+        <v>80</v>
+      </c>
+      <c r="J23">
+        <f>G23/I23*H23</f>
+        <v/>
       </c>
       <c r="K23" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Rebalance CabalArtilleryWalkerShell warheads and reload delays
Base shell: add missing ^HeavyCannon inherit (fixes orphaned warhead block),
Damage 8000->42000/class, Percentage 4->21, add FriendlyFire 21000 for
splash classes (Grenade, ShrapnelWeapon). 4 classes, H=0.9375.

Upgraded shell: same Damage/Percentage rebalance, add FriendlyFire for
MediumChemicalWeapon. 8 classes, H=1.0625. ReloadDelay stays 64 for both
(upgrade benefit = more classes = 13.3% higher DPS).

Spreadsheet row 2: G=42000, H=0.9375, I=64 (corrected from stale G=64000, H=1.125).
Formula: J=615.2, S=1272 (target 1250, within 2pct).
</commit_message>
<xml_diff>
--- a/docs/design/cameo_armor_system.xlsx
+++ b/docs/design/cameo_armor_system.xlsx
@@ -40786,16 +40786,17 @@
         <v>11.582</v>
       </c>
       <c r="G2" t="n">
-        <v>64000</v>
+        <v>42000</v>
       </c>
       <c r="H2" t="n">
-        <v>1.125</v>
+        <v>0.9375</v>
       </c>
       <c r="I2" t="n">
         <v>64</v>
       </c>
-      <c r="J2" t="n">
-        <v>1125</v>
+      <c r="J2">
+        <f>G2/I2*H2</f>
+        <v/>
       </c>
       <c r="K2" t="n">
         <v>1.25</v>

</xml_diff>